<commit_message>
feat: update uom product customer order
</commit_message>
<xml_diff>
--- a/Programming/WebFrontEnd/public/files/template-customer-order-product.xlsx
+++ b/Programming/WebFrontEnd/public/files/template-customer-order-product.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">No</t>
   </si>
@@ -41,9 +41,6 @@
   </si>
   <si>
     <t xml:space="preserve">Product Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UoM Name</t>
   </si>
   <si>
     <t xml:space="preserve">Qty</t>
@@ -351,11 +348,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1048576"/>
+  <dimension ref="A1:K1048576"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="27.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="4" style="1" width="27.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="4" style="1" width="27.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -391,9 +389,6 @@
       </c>
       <c r="K1" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -408,7 +403,6 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>